<commit_message>
feat: [special approval] update coo cc template & pdigt payment method
</commit_message>
<xml_diff>
--- a/src/assets/template/COO-CC-Template.xlsx
+++ b/src/assets/template/COO-CC-Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lin/Work/Philips/COS/COS-UI/src/assets/template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lin/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59654575-7FD8-8049-9F1F-DA0476CE0752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F450679D-BBC4-234A-9F95-7739B29605D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20500" xr2:uid="{54A4027A-E158-4545-81FE-CF92FEB69C28}"/>
   </bookViews>
@@ -197,7 +197,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="76">
   <si>
     <t>产品线</t>
   </si>
@@ -425,6 +425,14 @@
   </si>
   <si>
     <t>GCN</t>
+  </si>
+  <si>
+    <t>销售区域-Cycle Group</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>销售区域-Region</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -989,8 +997,8 @@
   <cols>
     <col min="1" max="1" width="10.83203125" style="14" customWidth="1"/>
     <col min="2" max="2" width="21" style="14" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" style="14" customWidth="1"/>
-    <col min="4" max="4" width="13.5" style="14" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" style="14" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" style="14" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" style="14" customWidth="1"/>
     <col min="6" max="6" width="16.5" style="14" customWidth="1"/>
     <col min="7" max="7" width="19.5" style="14" customWidth="1"/>
@@ -1025,10 +1033,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
fix: [special approval] COO issue
</commit_message>
<xml_diff>
--- a/src/assets/template/COO-CC-Template.xlsx
+++ b/src/assets/template/COO-CC-Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lin/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F450679D-BBC4-234A-9F95-7739B29605D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4288E20-D5CA-134C-BAD3-404964409F4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20500" xr2:uid="{54A4027A-E158-4545-81FE-CF92FEB69C28}"/>
+    <workbookView xWindow="42540" yWindow="100" windowWidth="35840" windowHeight="20500" xr2:uid="{54A4027A-E158-4545-81FE-CF92FEB69C28}"/>
   </bookViews>
   <sheets>
     <sheet name="10-1-3.COO CC Template" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,6 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={0C761EA7-99BF-46BB-9C10-AC5A273A4705}</author>
-    <author>tc={5D8A51A7-F5B9-41F9-8936-860ED28A885F}</author>
     <author>tc={BB884BC4-185B-4974-A4B0-8C8090B52839}</author>
     <author>tc={CA0BA64D-ADCB-4904-A5A8-FED7C98E989C}</author>
     <author>tc={F6A3E922-40A1-4EED-8801-F429B9DD9514}</author>
@@ -55,7 +54,7 @@
     add per requested</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{5D8A51A7-F5B9-41F9-8936-860ED28A885F}">
+    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{BB884BC4-185B-4974-A4B0-8C8090B52839}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -63,15 +62,7 @@
     add per requested</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="2" shapeId="0" xr:uid="{BB884BC4-185B-4974-A4B0-8C8090B52839}">
-      <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
-    add per requested</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="3" shapeId="0" xr:uid="{CA0BA64D-ADCB-4904-A5A8-FED7C98E989C}">
+    <comment ref="I1" authorId="2" shapeId="0" xr:uid="{CA0BA64D-ADCB-4904-A5A8-FED7C98E989C}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -79,7 +70,7 @@
     new add</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="4" shapeId="0" xr:uid="{F6A3E922-40A1-4EED-8801-F429B9DD9514}">
+    <comment ref="J1" authorId="3" shapeId="0" xr:uid="{F6A3E922-40A1-4EED-8801-F429B9DD9514}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -87,7 +78,7 @@
     new added</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="5" shapeId="0" xr:uid="{276688FF-4120-4383-B753-866264267731}">
+    <comment ref="M1" authorId="4" shapeId="0" xr:uid="{276688FF-4120-4383-B753-866264267731}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,7 +86,7 @@
     new add</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="6" shapeId="0" xr:uid="{153D344C-E0F8-4303-857C-C91D8C89C4F9}">
+    <comment ref="N1" authorId="5" shapeId="0" xr:uid="{153D344C-E0F8-4303-857C-C91D8C89C4F9}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -103,7 +94,7 @@
     和销售申请提供的SN号重复</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="7" shapeId="0" xr:uid="{298B914B-7BED-4362-B694-A981ADDF47B5}">
+    <comment ref="P1" authorId="6" shapeId="0" xr:uid="{298B914B-7BED-4362-B694-A981ADDF47B5}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -197,7 +188,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="77">
   <si>
     <t>产品线</t>
   </si>
@@ -432,6 +423,10 @@
   </si>
   <si>
     <t>销售区域-Region</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>保修期（月）</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -934,25 +929,22 @@
   <threadedComment ref="E1" dT="2022-02-15T08:29:11.72" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{0C761EA7-99BF-46BB-9C10-AC5A273A4705}">
     <text>add per requested</text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2022-02-15T08:29:11.72" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{5D8A51A7-F5B9-41F9-8936-860ED28A885F}">
+  <threadedComment ref="F1" dT="2022-02-15T08:29:11.72" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{BB884BC4-185B-4974-A4B0-8C8090B52839}">
     <text>add per requested</text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2022-02-15T08:29:11.72" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{BB884BC4-185B-4974-A4B0-8C8090B52839}">
-    <text>add per requested</text>
-  </threadedComment>
-  <threadedComment ref="J1" dT="2022-02-18T00:53:23.91" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{CA0BA64D-ADCB-4904-A5A8-FED7C98E989C}">
+  <threadedComment ref="I1" dT="2022-02-18T00:53:23.91" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{CA0BA64D-ADCB-4904-A5A8-FED7C98E989C}">
     <text>new add</text>
   </threadedComment>
-  <threadedComment ref="K1" dT="2022-03-11T00:12:24.57" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{F6A3E922-40A1-4EED-8801-F429B9DD9514}">
+  <threadedComment ref="J1" dT="2022-03-11T00:12:24.57" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{F6A3E922-40A1-4EED-8801-F429B9DD9514}">
     <text>new added</text>
   </threadedComment>
-  <threadedComment ref="N1" dT="2022-02-17T07:53:14.25" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{276688FF-4120-4383-B753-866264267731}">
+  <threadedComment ref="M1" dT="2022-02-17T07:53:14.25" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{276688FF-4120-4383-B753-866264267731}">
     <text>new add</text>
   </threadedComment>
-  <threadedComment ref="O1" dT="2022-03-17T05:34:48.64" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{153D344C-E0F8-4303-857C-C91D8C89C4F9}">
+  <threadedComment ref="N1" dT="2022-03-17T05:34:48.64" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{153D344C-E0F8-4303-857C-C91D8C89C4F9}">
     <text>和销售申请提供的SN号重复</text>
   </threadedComment>
-  <threadedComment ref="Q1" dT="2022-03-17T05:14:27.32" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{298B914B-7BED-4362-B694-A981ADDF47B5}">
+  <threadedComment ref="P1" dT="2022-03-17T05:14:27.32" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{298B914B-7BED-4362-B694-A981ADDF47B5}">
     <text>可否为月份？</text>
   </threadedComment>
 </ThreadedComments>
@@ -992,7 +984,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:Y9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="14" customWidth="1"/>
@@ -1000,32 +992,30 @@
     <col min="3" max="3" width="19.1640625" style="14" customWidth="1"/>
     <col min="4" max="4" width="14.6640625" style="14" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" style="14" customWidth="1"/>
-    <col min="6" max="6" width="16.5" style="14" customWidth="1"/>
-    <col min="7" max="7" width="19.5" style="14" customWidth="1"/>
-    <col min="8" max="8" width="25.33203125" style="14" customWidth="1"/>
-    <col min="9" max="9" width="22" style="14" customWidth="1"/>
-    <col min="10" max="10" width="10" style="14" customWidth="1"/>
-    <col min="11" max="11" width="10.5" style="14" customWidth="1"/>
-    <col min="12" max="12" width="15.5" style="14" customWidth="1"/>
-    <col min="13" max="13" width="16.1640625" style="14" customWidth="1"/>
-    <col min="14" max="14" width="20.1640625" style="14" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" style="14" customWidth="1"/>
-    <col min="16" max="16" width="13.5" style="14" customWidth="1"/>
-    <col min="17" max="17" width="19.83203125" style="17" customWidth="1"/>
-    <col min="18" max="18" width="16.5" style="17" customWidth="1"/>
-    <col min="19" max="19" width="16" style="17" customWidth="1"/>
-    <col min="20" max="20" width="19.5" style="17" customWidth="1"/>
-    <col min="21" max="21" width="15.5" style="14" customWidth="1"/>
-    <col min="22" max="22" width="17.6640625" style="14" customWidth="1"/>
-    <col min="23" max="23" width="20.83203125" style="14" customWidth="1"/>
-    <col min="24" max="24" width="16.33203125" style="14" customWidth="1"/>
-    <col min="25" max="25" width="14.83203125" style="14" customWidth="1"/>
-    <col min="26" max="26" width="17.5" style="14" customWidth="1"/>
-    <col min="27" max="27" width="19.6640625" style="14" customWidth="1"/>
-    <col min="28" max="16384" width="9.1640625" style="14"/>
+    <col min="6" max="6" width="19.5" style="14" customWidth="1"/>
+    <col min="7" max="7" width="25.33203125" style="14" customWidth="1"/>
+    <col min="8" max="8" width="22" style="14" customWidth="1"/>
+    <col min="9" max="9" width="10" style="14" customWidth="1"/>
+    <col min="10" max="10" width="10.5" style="14" customWidth="1"/>
+    <col min="11" max="11" width="15.5" style="14" customWidth="1"/>
+    <col min="12" max="12" width="16.1640625" style="14" customWidth="1"/>
+    <col min="13" max="13" width="20.1640625" style="14" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" style="14" customWidth="1"/>
+    <col min="15" max="15" width="13.5" style="14" customWidth="1"/>
+    <col min="16" max="16" width="19.83203125" style="17" customWidth="1"/>
+    <col min="17" max="17" width="16.5" style="17" customWidth="1"/>
+    <col min="18" max="18" width="19.5" style="17" customWidth="1"/>
+    <col min="19" max="19" width="15.5" style="14" customWidth="1"/>
+    <col min="20" max="20" width="17.6640625" style="14" customWidth="1"/>
+    <col min="21" max="21" width="20.83203125" style="14" customWidth="1"/>
+    <col min="22" max="22" width="16.33203125" style="14" customWidth="1"/>
+    <col min="23" max="23" width="14.83203125" style="14" customWidth="1"/>
+    <col min="24" max="24" width="17.5" style="14" customWidth="1"/>
+    <col min="25" max="25" width="19.6640625" style="14" customWidth="1"/>
+    <col min="26" max="16384" width="9.1640625" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="1" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1041,74 +1031,68 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
+      <c r="F1" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>10</v>
       </c>
+      <c r="K1" s="6" t="s">
+        <v>11</v>
+      </c>
       <c r="L1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="P1" s="6" t="s">
+        <v>16</v>
+      </c>
       <c r="Q1" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="T1" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="V1" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="W1" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="X1" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="Y1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:27" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="2" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1119,25 +1103,23 @@
       <c r="H2" s="8"/>
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
+      <c r="K2" s="9"/>
       <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="9"/>
+      <c r="O2" s="8"/>
+      <c r="P2" s="16"/>
       <c r="Q2" s="16"/>
       <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="T2" s="16"/>
+      <c r="S2" s="9"/>
+      <c r="T2" s="9"/>
       <c r="U2" s="9"/>
       <c r="V2" s="9"/>
       <c r="W2" s="9"/>
       <c r="X2" s="9"/>
       <c r="Y2" s="9"/>
-      <c r="Z2" s="9"/>
-      <c r="AA2" s="9"/>
-    </row>
-    <row r="3" spans="1:27" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="3" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -1148,25 +1130,23 @@
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
+      <c r="K3" s="9"/>
       <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="16"/>
       <c r="Q3" s="16"/>
       <c r="R3" s="16"/>
-      <c r="S3" s="16"/>
-      <c r="T3" s="16"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
       <c r="U3" s="9"/>
       <c r="V3" s="9"/>
       <c r="W3" s="9"/>
       <c r="X3" s="9"/>
       <c r="Y3" s="9"/>
-      <c r="Z3" s="9"/>
-      <c r="AA3" s="9"/>
-    </row>
-    <row r="4" spans="1:27" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="4" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -1177,25 +1157,23 @@
       <c r="H4" s="8"/>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
+      <c r="K4" s="9"/>
       <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="16"/>
       <c r="Q4" s="16"/>
       <c r="R4" s="16"/>
-      <c r="S4" s="16"/>
-      <c r="T4" s="16"/>
+      <c r="S4" s="9"/>
+      <c r="T4" s="9"/>
       <c r="U4" s="9"/>
       <c r="V4" s="9"/>
       <c r="W4" s="9"/>
       <c r="X4" s="9"/>
       <c r="Y4" s="9"/>
-      <c r="Z4" s="9"/>
-      <c r="AA4" s="9"/>
-    </row>
-    <row r="5" spans="1:27" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="5" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -1206,25 +1184,23 @@
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
+      <c r="K5" s="9"/>
       <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="16"/>
       <c r="Q5" s="16"/>
       <c r="R5" s="16"/>
-      <c r="S5" s="16"/>
-      <c r="T5" s="16"/>
+      <c r="S5" s="9"/>
+      <c r="T5" s="9"/>
       <c r="U5" s="9"/>
       <c r="V5" s="9"/>
       <c r="W5" s="9"/>
       <c r="X5" s="9"/>
       <c r="Y5" s="9"/>
-      <c r="Z5" s="9"/>
-      <c r="AA5" s="9"/>
-    </row>
-    <row r="6" spans="1:27" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="6" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -1235,25 +1211,23 @@
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
+      <c r="K6" s="9"/>
       <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="16"/>
       <c r="Q6" s="16"/>
       <c r="R6" s="16"/>
-      <c r="S6" s="16"/>
-      <c r="T6" s="16"/>
+      <c r="S6" s="9"/>
+      <c r="T6" s="9"/>
       <c r="U6" s="9"/>
       <c r="V6" s="9"/>
       <c r="W6" s="9"/>
       <c r="X6" s="9"/>
       <c r="Y6" s="9"/>
-      <c r="Z6" s="9"/>
-      <c r="AA6" s="9"/>
-    </row>
-    <row r="7" spans="1:27" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="7" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -1264,25 +1238,23 @@
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="K7" s="9"/>
       <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="16"/>
       <c r="Q7" s="16"/>
       <c r="R7" s="16"/>
-      <c r="S7" s="16"/>
-      <c r="T7" s="16"/>
+      <c r="S7" s="9"/>
+      <c r="T7" s="9"/>
       <c r="U7" s="9"/>
       <c r="V7" s="9"/>
       <c r="W7" s="9"/>
       <c r="X7" s="9"/>
       <c r="Y7" s="9"/>
-      <c r="Z7" s="9"/>
-      <c r="AA7" s="9"/>
-    </row>
-    <row r="8" spans="1:27" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="8" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -1293,25 +1265,23 @@
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
+      <c r="K8" s="9"/>
       <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="16"/>
       <c r="Q8" s="16"/>
       <c r="R8" s="16"/>
-      <c r="S8" s="16"/>
-      <c r="T8" s="16"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
       <c r="U8" s="9"/>
       <c r="V8" s="9"/>
       <c r="W8" s="9"/>
       <c r="X8" s="9"/>
       <c r="Y8" s="9"/>
-      <c r="Z8" s="9"/>
-      <c r="AA8" s="9"/>
-    </row>
-    <row r="9" spans="1:27" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="9" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -1322,23 +1292,21 @@
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
+      <c r="K9" s="9"/>
       <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="8"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="16"/>
       <c r="Q9" s="16"/>
       <c r="R9" s="16"/>
-      <c r="S9" s="16"/>
-      <c r="T9" s="16"/>
+      <c r="S9" s="9"/>
+      <c r="T9" s="9"/>
       <c r="U9" s="9"/>
       <c r="V9" s="9"/>
       <c r="W9" s="9"/>
       <c r="X9" s="9"/>
       <c r="Y9" s="9"/>
-      <c r="Z9" s="9"/>
-      <c r="AA9" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -1351,13 +1319,13 @@
           <x14:formula1>
             <xm:f>DropList!$K$5:$K$6</xm:f>
           </x14:formula1>
-          <xm:sqref>J2:J9</xm:sqref>
+          <xm:sqref>I2:I9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D985155F-0703-40E8-996F-6EF1A8D0055C}">
           <x14:formula1>
             <xm:f>DropList!$I$5:$I$6</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H9</xm:sqref>
+          <xm:sqref>G2:G9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EB0E75A2-12B1-4DED-B3F0-2B19294D4659}">
           <x14:formula1>
@@ -1381,19 +1349,19 @@
           <x14:formula1>
             <xm:f>DropList!$F$5:$F$6</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:F9</xm:sqref>
+          <xm:sqref>E2:E9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{145171C5-43EF-40FC-88F6-467CBA165051}">
           <x14:formula1>
             <xm:f>DropList!$V$5:$V$6</xm:f>
           </x14:formula1>
-          <xm:sqref>V2:V9</xm:sqref>
+          <xm:sqref>T2:T9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F97B1AFA-FE8C-4306-B545-9AA08A7DE8C0}">
           <x14:formula1>
             <xm:f>DropList!$W$5:$W$6</xm:f>
           </x14:formula1>
-          <xm:sqref>W2:W9</xm:sqref>
+          <xm:sqref>U2:U9</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
fix: [special approval] uat issue
</commit_message>
<xml_diff>
--- a/src/assets/template/COO-CC-Template.xlsx
+++ b/src/assets/template/COO-CC-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lin/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4288E20-D5CA-134C-BAD3-404964409F4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7353D694-2E4F-A940-B150-E2E3F24F65AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="42540" yWindow="100" windowWidth="35840" windowHeight="20500" xr2:uid="{54A4027A-E158-4545-81FE-CF92FEB69C28}"/>
   </bookViews>
@@ -46,7 +46,7 @@
     <author>tc={298B914B-7BED-4362-B694-A981ADDF47B5}</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{0C761EA7-99BF-46BB-9C10-AC5A273A4705}">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{0C761EA7-99BF-46BB-9C10-AC5A273A4705}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -54,7 +54,7 @@
     add per requested</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{BB884BC4-185B-4974-A4B0-8C8090B52839}">
+    <comment ref="E1" authorId="1" shapeId="0" xr:uid="{BB884BC4-185B-4974-A4B0-8C8090B52839}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -62,7 +62,7 @@
     add per requested</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="2" shapeId="0" xr:uid="{CA0BA64D-ADCB-4904-A5A8-FED7C98E989C}">
+    <comment ref="H1" authorId="2" shapeId="0" xr:uid="{CA0BA64D-ADCB-4904-A5A8-FED7C98E989C}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -70,7 +70,7 @@
     new add</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="3" shapeId="0" xr:uid="{F6A3E922-40A1-4EED-8801-F429B9DD9514}">
+    <comment ref="I1" authorId="3" shapeId="0" xr:uid="{F6A3E922-40A1-4EED-8801-F429B9DD9514}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -78,7 +78,7 @@
     new added</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="4" shapeId="0" xr:uid="{276688FF-4120-4383-B753-866264267731}">
+    <comment ref="L1" authorId="4" shapeId="0" xr:uid="{276688FF-4120-4383-B753-866264267731}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -86,7 +86,7 @@
     new add</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="5" shapeId="0" xr:uid="{153D344C-E0F8-4303-857C-C91D8C89C4F9}">
+    <comment ref="M1" authorId="5" shapeId="0" xr:uid="{153D344C-E0F8-4303-857C-C91D8C89C4F9}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -94,7 +94,7 @@
     和销售申请提供的SN号重复</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="6" shapeId="0" xr:uid="{298B914B-7BED-4362-B694-A981ADDF47B5}">
+    <comment ref="O1" authorId="6" shapeId="0" xr:uid="{298B914B-7BED-4362-B694-A981ADDF47B5}">
       <text>
         <t>[线程批注]
 你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
@@ -188,7 +188,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="77">
   <si>
     <t>产品线</t>
   </si>
@@ -926,25 +926,25 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="E1" dT="2022-02-15T08:29:11.72" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{0C761EA7-99BF-46BB-9C10-AC5A273A4705}">
+  <threadedComment ref="D1" dT="2022-02-15T08:29:11.72" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{0C761EA7-99BF-46BB-9C10-AC5A273A4705}">
     <text>add per requested</text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2022-02-15T08:29:11.72" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{BB884BC4-185B-4974-A4B0-8C8090B52839}">
+  <threadedComment ref="E1" dT="2022-02-15T08:29:11.72" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{BB884BC4-185B-4974-A4B0-8C8090B52839}">
     <text>add per requested</text>
   </threadedComment>
-  <threadedComment ref="I1" dT="2022-02-18T00:53:23.91" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{CA0BA64D-ADCB-4904-A5A8-FED7C98E989C}">
+  <threadedComment ref="H1" dT="2022-02-18T00:53:23.91" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{CA0BA64D-ADCB-4904-A5A8-FED7C98E989C}">
     <text>new add</text>
   </threadedComment>
-  <threadedComment ref="J1" dT="2022-03-11T00:12:24.57" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{F6A3E922-40A1-4EED-8801-F429B9DD9514}">
+  <threadedComment ref="I1" dT="2022-03-11T00:12:24.57" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{F6A3E922-40A1-4EED-8801-F429B9DD9514}">
     <text>new added</text>
   </threadedComment>
-  <threadedComment ref="M1" dT="2022-02-17T07:53:14.25" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{276688FF-4120-4383-B753-866264267731}">
+  <threadedComment ref="L1" dT="2022-02-17T07:53:14.25" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{276688FF-4120-4383-B753-866264267731}">
     <text>new add</text>
   </threadedComment>
-  <threadedComment ref="N1" dT="2022-03-17T05:34:48.64" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{153D344C-E0F8-4303-857C-C91D8C89C4F9}">
+  <threadedComment ref="M1" dT="2022-03-17T05:34:48.64" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{153D344C-E0F8-4303-857C-C91D8C89C4F9}">
     <text>和销售申请提供的SN号重复</text>
   </threadedComment>
-  <threadedComment ref="P1" dT="2022-03-17T05:14:27.32" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{298B914B-7BED-4362-B694-A981ADDF47B5}">
+  <threadedComment ref="O1" dT="2022-03-17T05:14:27.32" personId="{5DD14699-057C-4116-8E14-29413FC543F6}" id="{298B914B-7BED-4362-B694-A981ADDF47B5}">
     <text>可否为月份？</text>
   </threadedComment>
 </ThreadedComments>
@@ -984,115 +984,111 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:Y9"/>
+  <dimension ref="A1:X9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="14" customWidth="1"/>
-    <col min="2" max="2" width="21" style="14" customWidth="1"/>
-    <col min="3" max="3" width="19.1640625" style="14" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" style="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18" style="14" customWidth="1"/>
-    <col min="6" max="6" width="19.5" style="14" customWidth="1"/>
-    <col min="7" max="7" width="25.33203125" style="14" customWidth="1"/>
-    <col min="8" max="8" width="22" style="14" customWidth="1"/>
-    <col min="9" max="9" width="10" style="14" customWidth="1"/>
-    <col min="10" max="10" width="10.5" style="14" customWidth="1"/>
-    <col min="11" max="11" width="15.5" style="14" customWidth="1"/>
-    <col min="12" max="12" width="16.1640625" style="14" customWidth="1"/>
-    <col min="13" max="13" width="20.1640625" style="14" customWidth="1"/>
-    <col min="14" max="14" width="18.83203125" style="14" customWidth="1"/>
-    <col min="15" max="15" width="13.5" style="14" customWidth="1"/>
-    <col min="16" max="16" width="19.83203125" style="17" customWidth="1"/>
-    <col min="17" max="17" width="16.5" style="17" customWidth="1"/>
-    <col min="18" max="18" width="19.5" style="17" customWidth="1"/>
-    <col min="19" max="19" width="15.5" style="14" customWidth="1"/>
-    <col min="20" max="20" width="17.6640625" style="14" customWidth="1"/>
-    <col min="21" max="21" width="20.83203125" style="14" customWidth="1"/>
-    <col min="22" max="22" width="16.33203125" style="14" customWidth="1"/>
-    <col min="23" max="23" width="14.83203125" style="14" customWidth="1"/>
-    <col min="24" max="24" width="17.5" style="14" customWidth="1"/>
-    <col min="25" max="25" width="19.6640625" style="14" customWidth="1"/>
-    <col min="26" max="16384" width="9.1640625" style="14"/>
+    <col min="2" max="2" width="19.1640625" style="14" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" style="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" style="14" customWidth="1"/>
+    <col min="5" max="5" width="19.5" style="14" customWidth="1"/>
+    <col min="6" max="6" width="25.33203125" style="14" customWidth="1"/>
+    <col min="7" max="7" width="22" style="14" customWidth="1"/>
+    <col min="8" max="8" width="10" style="14" customWidth="1"/>
+    <col min="9" max="9" width="10.5" style="14" customWidth="1"/>
+    <col min="10" max="10" width="15.5" style="14" customWidth="1"/>
+    <col min="11" max="11" width="16.1640625" style="14" customWidth="1"/>
+    <col min="12" max="12" width="20.1640625" style="14" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" style="14" customWidth="1"/>
+    <col min="14" max="14" width="13.5" style="14" customWidth="1"/>
+    <col min="15" max="15" width="19.83203125" style="17" customWidth="1"/>
+    <col min="16" max="16" width="16.5" style="17" customWidth="1"/>
+    <col min="17" max="17" width="19.5" style="17" customWidth="1"/>
+    <col min="18" max="18" width="15.5" style="14" customWidth="1"/>
+    <col min="19" max="19" width="17.6640625" style="14" customWidth="1"/>
+    <col min="20" max="20" width="20.83203125" style="14" customWidth="1"/>
+    <col min="21" max="21" width="16.33203125" style="14" customWidth="1"/>
+    <col min="22" max="22" width="14.83203125" style="14" customWidth="1"/>
+    <col min="23" max="23" width="17.5" style="14" customWidth="1"/>
+    <col min="24" max="24" width="19.6640625" style="14" customWidth="1"/>
+    <col min="25" max="16384" width="9.1640625" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="1" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
+      <c r="B1" s="4" t="s">
+        <v>74</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" s="4" t="s">
         <v>75</v>
       </c>
+      <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
       <c r="E1" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>10</v>
       </c>
+      <c r="J1" s="6" t="s">
+        <v>11</v>
+      </c>
       <c r="K1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="L1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="O1" s="6" t="s">
+        <v>16</v>
+      </c>
       <c r="P1" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>19</v>
+        <v>76</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>76</v>
+        <v>21</v>
       </c>
       <c r="T1" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="V1" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="W1" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X1" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Y1" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="2" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1102,24 +1098,23 @@
       <c r="G2" s="8"/>
       <c r="H2" s="8"/>
       <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="J2" s="9"/>
       <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="9"/>
-      <c r="O2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="16"/>
       <c r="P2" s="16"/>
       <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
+      <c r="R2" s="9"/>
       <c r="S2" s="9"/>
       <c r="T2" s="9"/>
       <c r="U2" s="9"/>
       <c r="V2" s="9"/>
       <c r="W2" s="9"/>
       <c r="X2" s="9"/>
-      <c r="Y2" s="9"/>
-    </row>
-    <row r="3" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="3" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -1129,24 +1124,23 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
+      <c r="J3" s="9"/>
       <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="16"/>
       <c r="P3" s="16"/>
       <c r="Q3" s="16"/>
-      <c r="R3" s="16"/>
+      <c r="R3" s="9"/>
       <c r="S3" s="9"/>
       <c r="T3" s="9"/>
       <c r="U3" s="9"/>
       <c r="V3" s="9"/>
       <c r="W3" s="9"/>
       <c r="X3" s="9"/>
-      <c r="Y3" s="9"/>
-    </row>
-    <row r="4" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="4" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -1156,24 +1150,23 @@
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
       <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
+      <c r="J4" s="9"/>
       <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="8"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="16"/>
       <c r="P4" s="16"/>
       <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
+      <c r="R4" s="9"/>
       <c r="S4" s="9"/>
       <c r="T4" s="9"/>
       <c r="U4" s="9"/>
       <c r="V4" s="9"/>
       <c r="W4" s="9"/>
       <c r="X4" s="9"/>
-      <c r="Y4" s="9"/>
-    </row>
-    <row r="5" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="5" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -1183,24 +1176,23 @@
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
+      <c r="J5" s="9"/>
       <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="16"/>
       <c r="P5" s="16"/>
       <c r="Q5" s="16"/>
-      <c r="R5" s="16"/>
+      <c r="R5" s="9"/>
       <c r="S5" s="9"/>
       <c r="T5" s="9"/>
       <c r="U5" s="9"/>
       <c r="V5" s="9"/>
       <c r="W5" s="9"/>
       <c r="X5" s="9"/>
-      <c r="Y5" s="9"/>
-    </row>
-    <row r="6" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="6" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -1210,24 +1202,23 @@
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
+      <c r="J6" s="9"/>
       <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="16"/>
       <c r="P6" s="16"/>
       <c r="Q6" s="16"/>
-      <c r="R6" s="16"/>
+      <c r="R6" s="9"/>
       <c r="S6" s="9"/>
       <c r="T6" s="9"/>
       <c r="U6" s="9"/>
       <c r="V6" s="9"/>
       <c r="W6" s="9"/>
       <c r="X6" s="9"/>
-      <c r="Y6" s="9"/>
-    </row>
-    <row r="7" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="7" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -1237,24 +1228,23 @@
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
+      <c r="J7" s="9"/>
       <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="16"/>
       <c r="P7" s="16"/>
       <c r="Q7" s="16"/>
-      <c r="R7" s="16"/>
+      <c r="R7" s="9"/>
       <c r="S7" s="9"/>
       <c r="T7" s="9"/>
       <c r="U7" s="9"/>
       <c r="V7" s="9"/>
       <c r="W7" s="9"/>
       <c r="X7" s="9"/>
-      <c r="Y7" s="9"/>
-    </row>
-    <row r="8" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="8" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -1264,24 +1254,23 @@
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
+      <c r="J8" s="9"/>
       <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="16"/>
       <c r="P8" s="16"/>
       <c r="Q8" s="16"/>
-      <c r="R8" s="16"/>
+      <c r="R8" s="9"/>
       <c r="S8" s="9"/>
       <c r="T8" s="9"/>
       <c r="U8" s="9"/>
       <c r="V8" s="9"/>
       <c r="W8" s="9"/>
       <c r="X8" s="9"/>
-      <c r="Y8" s="9"/>
-    </row>
-    <row r="9" spans="1:25" s="7" customFormat="1" ht="25" customHeight="1">
+    </row>
+    <row r="9" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -1291,22 +1280,21 @@
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
+      <c r="J9" s="9"/>
       <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="8"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="16"/>
       <c r="P9" s="16"/>
       <c r="Q9" s="16"/>
-      <c r="R9" s="16"/>
+      <c r="R9" s="9"/>
       <c r="S9" s="9"/>
       <c r="T9" s="9"/>
       <c r="U9" s="9"/>
       <c r="V9" s="9"/>
       <c r="W9" s="9"/>
       <c r="X9" s="9"/>
-      <c r="Y9" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -1319,13 +1307,13 @@
           <x14:formula1>
             <xm:f>DropList!$K$5:$K$6</xm:f>
           </x14:formula1>
-          <xm:sqref>I2:I9</xm:sqref>
+          <xm:sqref>H2:H9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D985155F-0703-40E8-996F-6EF1A8D0055C}">
           <x14:formula1>
             <xm:f>DropList!$I$5:$I$6</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G9</xm:sqref>
+          <xm:sqref>F2:F9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EB0E75A2-12B1-4DED-B3F0-2B19294D4659}">
           <x14:formula1>
@@ -1337,31 +1325,31 @@
           <x14:formula1>
             <xm:f>DropList!$E$5:$E$13</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D9</xm:sqref>
+          <xm:sqref>C2:C9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{56AC1C1C-EA51-46E1-81EA-2B3DE656F9DA}">
           <x14:formula1>
             <xm:f>DropList!$D$5:$D$9</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C9</xm:sqref>
+          <xm:sqref>B2:B9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4D39DB34-78CD-4B51-B0C7-2C15E2B8F5CA}">
           <x14:formula1>
             <xm:f>DropList!$F$5:$F$6</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E9</xm:sqref>
+          <xm:sqref>D2:D9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{145171C5-43EF-40FC-88F6-467CBA165051}">
           <x14:formula1>
             <xm:f>DropList!$V$5:$V$6</xm:f>
           </x14:formula1>
-          <xm:sqref>T2:T9</xm:sqref>
+          <xm:sqref>S2:S9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F97B1AFA-FE8C-4306-B545-9AA08A7DE8C0}">
           <x14:formula1>
             <xm:f>DropList!$W$5:$W$6</xm:f>
           </x14:formula1>
-          <xm:sqref>U2:U9</xm:sqref>
+          <xm:sqref>T2:T9</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
fix[special approval]: coo cc import date issue
</commit_message>
<xml_diff>
--- a/src/assets/template/COO-CC-Template.xlsx
+++ b/src/assets/template/COO-CC-Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11010"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lin/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Project\Philips\COS\COS-UI\src\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7353D694-2E4F-A940-B150-E2E3F24F65AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{675CC5EB-E846-4DF1-AED7-AA16D14C336B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42540" yWindow="100" windowWidth="35840" windowHeight="20500" xr2:uid="{54A4027A-E158-4545-81FE-CF92FEB69C28}"/>
+    <workbookView xWindow="-30828" yWindow="-4248" windowWidth="30936" windowHeight="16896" xr2:uid="{54A4027A-E158-4545-81FE-CF92FEB69C28}"/>
   </bookViews>
   <sheets>
     <sheet name="10-1-3.COO CC Template" sheetId="1" r:id="rId1"/>
@@ -48,57 +48,57 @@
   <commentList>
     <comment ref="D1" authorId="0" shapeId="0" xr:uid="{0C761EA7-99BF-46BB-9C10-AC5A273A4705}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     add per requested</t>
       </text>
     </comment>
     <comment ref="E1" authorId="1" shapeId="0" xr:uid="{BB884BC4-185B-4974-A4B0-8C8090B52839}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     add per requested</t>
       </text>
     </comment>
     <comment ref="H1" authorId="2" shapeId="0" xr:uid="{CA0BA64D-ADCB-4904-A5A8-FED7C98E989C}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     new add</t>
       </text>
     </comment>
     <comment ref="I1" authorId="3" shapeId="0" xr:uid="{F6A3E922-40A1-4EED-8801-F429B9DD9514}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     new added</t>
       </text>
     </comment>
     <comment ref="L1" authorId="4" shapeId="0" xr:uid="{276688FF-4120-4383-B753-866264267731}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     new add</t>
       </text>
     </comment>
     <comment ref="M1" authorId="5" shapeId="0" xr:uid="{153D344C-E0F8-4303-857C-C91D8C89C4F9}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     和销售申请提供的SN号重复</t>
       </text>
     </comment>
     <comment ref="O1" authorId="6" shapeId="0" xr:uid="{298B914B-7BED-4362-B694-A981ADDF47B5}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     可否为月份？</t>
       </text>
     </comment>
@@ -121,65 +121,65 @@
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0" xr:uid="{01E7279A-D807-40BA-968C-75850356F51E}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     add per requested</t>
       </text>
     </comment>
     <comment ref="F1" authorId="1" shapeId="0" xr:uid="{87D50B8F-A819-4D99-B085-F2DF2F0ABDBF}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     add per requested</t>
       </text>
     </comment>
     <comment ref="G1" authorId="2" shapeId="0" xr:uid="{FCDFAAC5-D430-40B3-9EA0-E84342B090C5}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     add per requested</t>
       </text>
     </comment>
     <comment ref="J1" authorId="3" shapeId="0" xr:uid="{77EB2245-B06F-4DE1-B745-711E565591A5}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     new add</t>
       </text>
     </comment>
     <comment ref="K1" authorId="4" shapeId="0" xr:uid="{AACFB746-997C-4E6A-904D-FB51491AFAFA}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     new added</t>
       </text>
     </comment>
     <comment ref="N1" authorId="5" shapeId="0" xr:uid="{8303A5E6-A2BA-4A21-8131-297072CA26CD}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     new add</t>
       </text>
     </comment>
     <comment ref="O1" authorId="6" shapeId="0" xr:uid="{64B0E3F6-D027-47D3-8CCE-B0F328308836}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     和销售申请提供的SN号重复</t>
       </text>
     </comment>
     <comment ref="Q1" authorId="7" shapeId="0" xr:uid="{9975895D-DA5D-47D0-A6F9-85FB74DF56F0}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     可否为月份？</t>
       </text>
     </comment>
@@ -434,35 +434,36 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="0"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color indexed="8"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -470,13 +471,13 @@
       <b/>
       <sz val="10"/>
       <color indexed="8"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -588,7 +589,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -600,15 +601,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -630,7 +631,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -985,36 +986,36 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:X9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="25" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="25.05" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="14" customWidth="1"/>
-    <col min="2" max="2" width="19.1640625" style="14" customWidth="1"/>
+    <col min="1" max="1" width="10.77734375" style="14" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" style="14" customWidth="1"/>
     <col min="3" max="3" width="14.6640625" style="14" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" style="14" customWidth="1"/>
-    <col min="5" max="5" width="19.5" style="14" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" style="14" customWidth="1"/>
     <col min="6" max="6" width="25.33203125" style="14" customWidth="1"/>
     <col min="7" max="7" width="22" style="14" customWidth="1"/>
     <col min="8" max="8" width="10" style="14" customWidth="1"/>
-    <col min="9" max="9" width="10.5" style="14" customWidth="1"/>
-    <col min="10" max="10" width="15.5" style="14" customWidth="1"/>
-    <col min="11" max="11" width="16.1640625" style="14" customWidth="1"/>
-    <col min="12" max="12" width="20.1640625" style="14" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" style="14" customWidth="1"/>
-    <col min="14" max="14" width="13.5" style="14" customWidth="1"/>
-    <col min="15" max="15" width="19.83203125" style="17" customWidth="1"/>
-    <col min="16" max="16" width="16.5" style="17" customWidth="1"/>
-    <col min="17" max="17" width="19.5" style="17" customWidth="1"/>
-    <col min="18" max="18" width="15.5" style="14" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" style="14" customWidth="1"/>
+    <col min="10" max="10" width="15.44140625" style="14" customWidth="1"/>
+    <col min="11" max="11" width="16.109375" style="14" customWidth="1"/>
+    <col min="12" max="12" width="20.109375" style="14" customWidth="1"/>
+    <col min="13" max="13" width="18.77734375" style="14" customWidth="1"/>
+    <col min="14" max="14" width="13.44140625" style="14" customWidth="1"/>
+    <col min="15" max="15" width="19.77734375" style="17" customWidth="1"/>
+    <col min="16" max="16" width="16.44140625" style="17" customWidth="1"/>
+    <col min="17" max="17" width="19.44140625" style="17" customWidth="1"/>
+    <col min="18" max="18" width="15.44140625" style="14" customWidth="1"/>
     <col min="19" max="19" width="17.6640625" style="14" customWidth="1"/>
-    <col min="20" max="20" width="20.83203125" style="14" customWidth="1"/>
+    <col min="20" max="20" width="20.77734375" style="14" customWidth="1"/>
     <col min="21" max="21" width="16.33203125" style="14" customWidth="1"/>
-    <col min="22" max="22" width="14.83203125" style="14" customWidth="1"/>
-    <col min="23" max="23" width="17.5" style="14" customWidth="1"/>
+    <col min="22" max="22" width="14.77734375" style="14" customWidth="1"/>
+    <col min="23" max="23" width="17.44140625" style="14" customWidth="1"/>
     <col min="24" max="24" width="19.6640625" style="14" customWidth="1"/>
-    <col min="25" max="16384" width="9.1640625" style="14"/>
+    <col min="25" max="16384" width="9.109375" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="1" spans="1:24" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1088,7 +1089,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="2" spans="1:24" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1114,7 +1115,7 @@
       <c r="W2" s="9"/>
       <c r="X2" s="9"/>
     </row>
-    <row r="3" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="3" spans="1:24" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -1140,7 +1141,7 @@
       <c r="W3" s="9"/>
       <c r="X3" s="9"/>
     </row>
-    <row r="4" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="4" spans="1:24" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -1166,7 +1167,7 @@
       <c r="W4" s="9"/>
       <c r="X4" s="9"/>
     </row>
-    <row r="5" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="5" spans="1:24" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -1192,7 +1193,7 @@
       <c r="W5" s="9"/>
       <c r="X5" s="9"/>
     </row>
-    <row r="6" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="6" spans="1:24" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -1218,7 +1219,7 @@
       <c r="W6" s="9"/>
       <c r="X6" s="9"/>
     </row>
-    <row r="7" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="7" spans="1:24" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -1244,7 +1245,7 @@
       <c r="W7" s="9"/>
       <c r="X7" s="9"/>
     </row>
-    <row r="8" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="8" spans="1:24" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -1270,7 +1271,7 @@
       <c r="W8" s="9"/>
       <c r="X8" s="9"/>
     </row>
-    <row r="9" spans="1:24" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="9" spans="1:24" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -1360,9 +1361,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AF8FCDC-D816-421C-B55D-46F569A12CAC}">
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:28" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="1" spans="1:28" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1445,7 +1446,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="2" spans="1:28" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
@@ -1529,7 +1530,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="3" spans="1:28" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>36</v>
       </c>
@@ -1585,7 +1586,7 @@
       <c r="AA3" s="11"/>
       <c r="AB3" s="11"/>
     </row>
-    <row r="4" spans="1:28" s="7" customFormat="1" ht="25" customHeight="1">
+    <row r="4" spans="1:28" s="7" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>49</v>
       </c>
@@ -1671,7 +1672,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="14" customFormat="1" ht="25" customHeight="1">
+    <row r="5" spans="1:28" s="14" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="13" t="s">
         <v>55</v>
       </c>
@@ -1703,7 +1704,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="14" customFormat="1" ht="25" customHeight="1">
+    <row r="6" spans="1:28" s="14" customFormat="1" ht="25.05" customHeight="1">
       <c r="B6" s="14" t="s">
         <v>62</v>
       </c>
@@ -1729,7 +1730,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="14" customFormat="1" ht="25" customHeight="1">
+    <row r="7" spans="1:28" s="14" customFormat="1" ht="25.05" customHeight="1">
       <c r="B7" s="14" t="s">
         <v>27</v>
       </c>
@@ -1740,7 +1741,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="14" customFormat="1" ht="25" customHeight="1">
+    <row r="8" spans="1:28" s="14" customFormat="1" ht="25.05" customHeight="1">
       <c r="B8" s="14" t="s">
         <v>69</v>
       </c>
@@ -1751,7 +1752,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="14" customFormat="1" ht="25" customHeight="1">
+    <row r="9" spans="1:28" s="14" customFormat="1" ht="25.05" customHeight="1">
       <c r="B9" s="14" t="s">
         <v>71</v>
       </c>
@@ -1762,22 +1763,22 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="14" customFormat="1" ht="25" customHeight="1">
+    <row r="10" spans="1:28" s="14" customFormat="1" ht="25.05" customHeight="1">
       <c r="E10" s="14" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="14" customFormat="1" ht="25" customHeight="1">
+    <row r="11" spans="1:28" s="14" customFormat="1" ht="25.05" customHeight="1">
       <c r="E11" s="14" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="14" customFormat="1" ht="25" customHeight="1">
+    <row r="12" spans="1:28" s="14" customFormat="1" ht="25.05" customHeight="1">
       <c r="E12" s="14" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="14" customFormat="1" ht="25" customHeight="1">
+    <row r="13" spans="1:28" s="14" customFormat="1" ht="25.05" customHeight="1">
       <c r="E13" s="14" t="s">
         <v>71</v>
       </c>

</xml_diff>